<commit_message>
docs: record confirmed invoice defect
</commit_message>
<xml_diff>
--- a/Report Test subject/defects/exports/OSMS-Defect-Log.xlsx
+++ b/Report Test subject/defects/exports/OSMS-Defect-Log.xlsx
@@ -8,35 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\Online-Sales-Management-System\Report Test subject\defects\exports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF5B7AA9-AAE1-4499-8525-FE04A3497191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8737A264-8EA9-49A9-B6E4-7EF737F27239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9D56C048-253C-4B39-A445-84BECE6AAB45}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C7E08124-F172-4617-B2D8-E0D19190FF5A}"/>
   </bookViews>
   <sheets>
-    <sheet name="DefectLog" sheetId="1" r:id="rId1"/>
+    <sheet name="OSMS-Defect-Register" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="58">
   <si>
     <t>Record ID</t>
   </si>
@@ -116,25 +100,25 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>Pending Manual Confirmation</t>
-  </si>
-  <si>
-    <t>Sales user account is available and UI automation runner is configured</t>
-  </si>
-  <si>
-    <t>1. Execute the filtered UI automation run containing SalesUserIsDeniedAccessToPurchases. 2. Allow the test to navigate after login. 3. Observe the final page state and runner timeout.</t>
-  </si>
-  <si>
-    <t>Sales user should be denied access to the Purchases area according to the intended permission rule</t>
-  </si>
-  <si>
-    <t>Automation timed out while waiting for an access-denied state and the screenshot shows sales@osms.local on the dashboard instead of a confirmed denial page</t>
-  </si>
-  <si>
-    <t>evidence/ui/automation/20260405_115343_TC-UI-AUTH-003-failure.png ; results/automation-ui/ui-tests.trx</t>
-  </si>
-  <si>
-    <t>Do not open as a product defect until manual reproduction confirms an authorization problem</t>
+    <t>Closed - Behavior Confirmed</t>
+  </si>
+  <si>
+    <t>Sales user account is available and focused UI rerun is configured.</t>
+  </si>
+  <si>
+    <t>1. Log in as sales@osms.local. 2. Navigate directly to /Admin/Purchases. 3. Observe the resulting page and route.</t>
+  </si>
+  <si>
+    <t>Sales user should be denied access to Purchases by an equivalent permission-denial behavior.</t>
+  </si>
+  <si>
+    <t>The app returned a denial by redirecting the sales user away from /Admin/Purchases to the dashboard. This matched the denial intent, so no product defect remains.</t>
+  </si>
+  <si>
+    <t>evidence/ui/automation/20260406_054245_TC-UI-AUTH-003-access-denied.png ; results/automation-ui/auth-permission-rerun.trx</t>
+  </si>
+  <si>
+    <t>Original timeout was an automation expectation mismatch, not a product defect.</t>
   </si>
   <si>
     <t>OBS-20260405-002</t>
@@ -146,29 +130,77 @@
     <t>Products Import</t>
   </si>
   <si>
-    <t>Warehouse account is available and the mixed-validation workbook exists</t>
-  </si>
-  <si>
-    <t>1. Execute the filtered UI automation run containing ProductImportPreviewShowsExpectedValidAndInvalidCounts. 2. Upload OSMS-Product-Import-Mixed-Validation.xlsx. 3. Observe the interaction with the preview action.</t>
-  </si>
-  <si>
-    <t>The import preview should proceed and display valid and invalid row counts for the uploaded workbook</t>
-  </si>
-  <si>
-    <t>Automation timed out before the preview interaction completed and the screenshot only proves the workbook was selected on the import page</t>
-  </si>
-  <si>
-    <t>evidence/ui/automation/20260405_115405_TC-UI-IMP-002-failure.png ; results/automation-ui/ui-tests.trx</t>
-  </si>
-  <si>
-    <t>Do not open as a product defect until manual reproduction confirms a broken import-preview flow</t>
+    <t>Closed - Automation Fixed</t>
+  </si>
+  <si>
+    <t>Warehouse account is available and the mixed-validation workbook exists.</t>
+  </si>
+  <si>
+    <t>1. Log in as warehouse@osms.local. 2. Open /Admin/Products/ImportExcel. 3. Upload OSMS-Product-Import-Mixed-Validation.xlsx and preview it.</t>
+  </si>
+  <si>
+    <t>The preview should open and display summary counts for valid and invalid rows.</t>
+  </si>
+  <si>
+    <t>The focused rerun passed after narrowing the submit locator to the correct import form. The application behavior is now confirmed working for this case.</t>
+  </si>
+  <si>
+    <t>evidence/ui/automation/20260406_054115_TC-UI-IMP-002-preview.png ; results/automation-ui/import-preview-rerun.trx</t>
+  </si>
+  <si>
+    <t>Original timeout came from a broad submit locator in automation, not a confirmed product defect.</t>
+  </si>
+  <si>
+    <t>BUG-20260406-001</t>
+  </si>
+  <si>
+    <t>Confirmed Defect</t>
+  </si>
+  <si>
+    <t>TC-UI-INV-001</t>
+  </si>
+  <si>
+    <t>Invoices</t>
+  </si>
+  <si>
+    <t>UI + Server Log</t>
+  </si>
+  <si>
+    <t>http://localhost:5068 + Chrome headless via Selenium xUnit + ASP.NET Core server log</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Open - Confirmed</t>
+  </si>
+  <si>
+    <t>PENDING REAL EXECUTION - GitHub CLI unavailable in local environment</t>
+  </si>
+  <si>
+    <t>Admin user is logged in; invoice create page is reachable; active product SP010 with stock is available.</t>
+  </si>
+  <si>
+    <t>1. Log in as admin@osms.local. 2. Open /Admin/Invoices/Create. 3. Leave customer as walk-in. 4. Select SP010 with quantity 1. 5. Submit the invoice.</t>
+  </si>
+  <si>
+    <t>A new invoice should be created successfully, stock should be reduced, and the user should be redirected to the invoice details page.</t>
+  </si>
+  <si>
+    <t>The create action stays on the Create page and shows the toast Failed to create invoice. Please check data and try again. The server log confirms InvalidOperationException from MySqlRetryingExecutionStrategy when a user-initiated transaction is started in InvoicesController.Create.</t>
+  </si>
+  <si>
+    <t>evidence/ui/automation/20260406_053902_TC-UI-INV-001-failure.png ; results/automation-ui/invoice-rerun.trx ; evidence/defects/BUG-20260406-001-invoice-create-log.txt</t>
+  </si>
+  <si>
+    <t>Confirmed defect because both UI behavior and server-side exception are reproducible in the current environment.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="14"/>
       <color theme="1"/>
@@ -176,16 +208,317 @@
       <family val="2"/>
       <charset val="163"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+      <charset val="163"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF006100"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF9C0006"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF9C5700"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -193,16 +526,205 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="42">
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -533,29 +1055,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64DA97FF-D436-4659-BA9C-2834BB4BE3C0}">
-  <dimension ref="A1:R3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BB41EA0-38BD-4E8A-9245-0374C8BE6D8A}">
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="51.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="63.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="191.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="89.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="136.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="91.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="84.5546875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -701,31 +1203,87 @@
         <v>25</v>
       </c>
       <c r="K3" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="L3" t="s">
         <v>25</v>
       </c>
       <c r="M3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="R3" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="1">
+        <v>46118</v>
+      </c>
+      <c r="D4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K4" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" t="s">
+        <v>52</v>
+      </c>
+      <c r="N4" t="s">
+        <v>53</v>
+      </c>
+      <c r="O4" t="s">
+        <v>54</v>
+      </c>
+      <c r="P4" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>56</v>
+      </c>
+      <c r="R4" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>